<commit_message>
Add Seggregate0sand1s.java to implement array segregation of 0s and 1s
</commit_message>
<xml_diff>
--- a/DSA patterns Cheat Sheet.xlsx
+++ b/DSA patterns Cheat Sheet.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="373">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2149,15 +2149,15 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -2870,19 +2870,19 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1"/>
   </cellXfs>
@@ -3432,19 +3432,22 @@
       </c>
       <c r="D5" s="14"/>
       <c r="E5" s="15"/>
+      <c r="F5" s="12" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="6" customHeight="1" spans="1:6">
       <c r="A6" s="8"/>
       <c r="B6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="16" t="s">
         <v>16</v>
       </c>
       <c r="F6" s="12" t="s">
@@ -3456,7 +3459,7 @@
       <c r="B7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="18" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="11"/>
@@ -3470,7 +3473,7 @@
       <c r="B8" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="16" t="s">
         <v>20</v>
       </c>
       <c r="D8" s="11"/>
@@ -3484,7 +3487,7 @@
       <c r="B9" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="16" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="11"/>
@@ -3498,7 +3501,7 @@
       <c r="B10" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="13" t="s">
         <v>24</v>
       </c>
       <c r="D10" s="11"/>
@@ -3512,7 +3515,7 @@
       <c r="B11" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="16" t="s">
         <v>26</v>
       </c>
       <c r="D11" s="11"/>
@@ -3528,13 +3531,16 @@
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="11"/>
+      <c r="F12" s="12" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="13" customHeight="1" spans="1:6">
       <c r="A13" s="8"/>
       <c r="B13" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="16" t="s">
         <v>30</v>
       </c>
       <c r="D13" s="11"/>
@@ -3545,7 +3551,7 @@
       <c r="B14" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="16" t="s">
         <v>32</v>
       </c>
       <c r="D14" s="11"/>
@@ -3556,10 +3562,10 @@
       <c r="B15" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="16" t="s">
         <v>35</v>
       </c>
     </row>
@@ -3577,7 +3583,7 @@
       <c r="B17" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="16" t="s">
         <v>38</v>
       </c>
       <c r="D17" s="11"/>
@@ -3588,7 +3594,7 @@
       <c r="B18" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="16" t="s">
         <v>40</v>
       </c>
       <c r="D18" s="11"/>
@@ -3599,7 +3605,7 @@
       <c r="B19" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="16" t="s">
         <v>42</v>
       </c>
       <c r="D19" s="11"/>
@@ -3610,7 +3616,7 @@
       <c r="B20" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D20" s="11"/>
@@ -3621,7 +3627,7 @@
       <c r="B21" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="16" t="s">
         <v>46</v>
       </c>
       <c r="D21" s="11"/>
@@ -3632,7 +3638,7 @@
       <c r="B22" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="16" t="s">
         <v>48</v>
       </c>
       <c r="D22" s="11"/>
@@ -3643,7 +3649,7 @@
       <c r="B23" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="16" t="s">
         <v>50</v>
       </c>
       <c r="D23" s="11"/>
@@ -3654,7 +3660,7 @@
       <c r="B24" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="16" t="s">
         <v>52</v>
       </c>
       <c r="D24" s="11"/>
@@ -3685,7 +3691,7 @@
       <c r="B27" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="16" t="s">
         <v>57</v>
       </c>
       <c r="D27" s="11"/>
@@ -3696,7 +3702,7 @@
       <c r="B28" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="16" t="s">
         <v>59</v>
       </c>
       <c r="D28" s="11"/>
@@ -3707,7 +3713,7 @@
       <c r="B29" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="16" t="s">
         <v>61</v>
       </c>
       <c r="D29" s="11"/>
@@ -3718,7 +3724,7 @@
       <c r="B30" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C30" s="16" t="s">
         <v>63</v>
       </c>
       <c r="D30" s="11"/>
@@ -3729,7 +3735,7 @@
       <c r="B31" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="16" t="s">
         <v>65</v>
       </c>
       <c r="D31" s="11"/>
@@ -3740,7 +3746,7 @@
       <c r="B32" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C32" s="16" t="s">
         <v>67</v>
       </c>
       <c r="D32" s="11"/>
@@ -3751,7 +3757,7 @@
       <c r="B33" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="16" t="s">
         <v>57</v>
       </c>
       <c r="D33" s="11"/>
@@ -3762,7 +3768,7 @@
       <c r="B34" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="16" t="s">
         <v>70</v>
       </c>
       <c r="D34" s="11"/>
@@ -3773,7 +3779,7 @@
       <c r="B35" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="C35" s="13" t="s">
+      <c r="C35" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D35" s="11"/>
@@ -3784,7 +3790,7 @@
       <c r="B36" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C36" s="16" t="s">
         <v>74</v>
       </c>
       <c r="D36" s="11"/>
@@ -3795,7 +3801,7 @@
       <c r="B37" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C37" s="17" t="s">
+      <c r="C37" s="18" t="s">
         <v>76</v>
       </c>
       <c r="D37" s="11"/>
@@ -3965,7 +3971,7 @@
       <c r="B53" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="C53" s="13" t="s">
+      <c r="C53" s="16" t="s">
         <v>105</v>
       </c>
       <c r="D53" s="11"/>
@@ -3976,7 +3982,7 @@
       <c r="B54" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C54" s="13" t="s">
+      <c r="C54" s="16" t="s">
         <v>107</v>
       </c>
       <c r="D54" s="11"/>
@@ -3987,7 +3993,7 @@
       <c r="B55" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="C55" s="13" t="s">
+      <c r="C55" s="16" t="s">
         <v>109</v>
       </c>
       <c r="D55" s="11"/>
@@ -3998,7 +4004,7 @@
       <c r="B56" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="C56" s="13" t="s">
+      <c r="C56" s="16" t="s">
         <v>111</v>
       </c>
       <c r="E56" s="11"/>
@@ -4008,7 +4014,7 @@
       <c r="B57" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="C57" s="13" t="s">
+      <c r="C57" s="16" t="s">
         <v>113</v>
       </c>
       <c r="D57" s="11"/>
@@ -4019,7 +4025,7 @@
       <c r="B58" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="C58" s="13" t="s">
+      <c r="C58" s="16" t="s">
         <v>115</v>
       </c>
       <c r="D58" s="11"/>
@@ -4030,7 +4036,7 @@
       <c r="B59" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="C59" s="13" t="s">
+      <c r="C59" s="16" t="s">
         <v>117</v>
       </c>
       <c r="D59" s="11"/>
@@ -4050,7 +4056,7 @@
       <c r="B61" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="C61" s="13" t="s">
+      <c r="C61" s="16" t="s">
         <v>120</v>
       </c>
       <c r="E61" s="11"/>
@@ -4060,7 +4066,7 @@
       <c r="B62" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="C62" s="13" t="s">
+      <c r="C62" s="16" t="s">
         <v>122</v>
       </c>
       <c r="D62" s="11"/>
@@ -4071,7 +4077,7 @@
       <c r="B63" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="C63" s="13" t="s">
+      <c r="C63" s="16" t="s">
         <v>124</v>
       </c>
       <c r="D63" s="11"/>
@@ -4082,7 +4088,7 @@
       <c r="B64" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="C64" s="13" t="s">
+      <c r="C64" s="16" t="s">
         <v>126</v>
       </c>
       <c r="D64" s="11"/>
@@ -4093,7 +4099,7 @@
       <c r="B65" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="C65" s="13" t="s">
+      <c r="C65" s="16" t="s">
         <v>128</v>
       </c>
       <c r="D65" s="11"/>
@@ -4104,7 +4110,7 @@
       <c r="B66" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="C66" s="13" t="s">
+      <c r="C66" s="16" t="s">
         <v>130</v>
       </c>
       <c r="D66" s="11"/>
@@ -4115,7 +4121,7 @@
       <c r="B67" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="C67" s="13" t="s">
+      <c r="C67" s="16" t="s">
         <v>132</v>
       </c>
       <c r="D67" s="11"/>
@@ -4126,7 +4132,7 @@
       <c r="B68" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="C68" s="13" t="s">
+      <c r="C68" s="16" t="s">
         <v>134</v>
       </c>
       <c r="D68" s="11"/>
@@ -4146,7 +4152,7 @@
       <c r="B70" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="C70" s="13" t="s">
+      <c r="C70" s="16" t="s">
         <v>137</v>
       </c>
       <c r="D70" s="11"/>
@@ -4157,7 +4163,7 @@
       <c r="B71" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="C71" s="13" t="s">
+      <c r="C71" s="16" t="s">
         <v>139</v>
       </c>
       <c r="D71" s="11"/>
@@ -4168,7 +4174,7 @@
       <c r="B72" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="C72" s="13" t="s">
+      <c r="C72" s="16" t="s">
         <v>141</v>
       </c>
       <c r="D72" s="11"/>
@@ -4179,7 +4185,7 @@
       <c r="B73" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="C73" s="13" t="s">
+      <c r="C73" s="16" t="s">
         <v>143</v>
       </c>
       <c r="D73" s="11"/>
@@ -4190,7 +4196,7 @@
       <c r="B74" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="C74" s="13" t="s">
+      <c r="C74" s="16" t="s">
         <v>145</v>
       </c>
       <c r="D74" s="11"/>
@@ -4201,7 +4207,7 @@
       <c r="B75" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="C75" s="13" t="s">
+      <c r="C75" s="16" t="s">
         <v>147</v>
       </c>
       <c r="D75" s="11"/>
@@ -4221,7 +4227,7 @@
       <c r="B77" s="24" t="s">
         <v>149</v>
       </c>
-      <c r="C77" s="13" t="s">
+      <c r="C77" s="16" t="s">
         <v>150</v>
       </c>
       <c r="D77" s="11"/>
@@ -4232,7 +4238,7 @@
       <c r="B78" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="C78" s="13" t="s">
+      <c r="C78" s="16" t="s">
         <v>152</v>
       </c>
       <c r="D78" s="11"/>
@@ -4252,7 +4258,7 @@
       <c r="B80" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="C80" s="13" t="s">
+      <c r="C80" s="16" t="s">
         <v>155</v>
       </c>
       <c r="D80" s="15"/>
@@ -4263,7 +4269,7 @@
       <c r="B81" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="C81" s="13" t="s">
+      <c r="C81" s="16" t="s">
         <v>157</v>
       </c>
       <c r="D81" s="11"/>
@@ -4274,7 +4280,7 @@
       <c r="B82" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="C82" s="13" t="s">
+      <c r="C82" s="16" t="s">
         <v>159</v>
       </c>
       <c r="D82" s="11"/>
@@ -4285,7 +4291,7 @@
       <c r="B83" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="C83" s="13" t="s">
+      <c r="C83" s="16" t="s">
         <v>161</v>
       </c>
       <c r="D83" s="11"/>
@@ -4296,7 +4302,7 @@
       <c r="B84" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="C84" s="13" t="s">
+      <c r="C84" s="16" t="s">
         <v>163</v>
       </c>
       <c r="D84" s="11"/>
@@ -4307,7 +4313,7 @@
       <c r="B85" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="C85" s="13" t="s">
+      <c r="C85" s="16" t="s">
         <v>165</v>
       </c>
       <c r="D85" s="11"/>
@@ -4327,7 +4333,7 @@
       <c r="B87" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="C87" s="13" t="s">
+      <c r="C87" s="16" t="s">
         <v>168</v>
       </c>
       <c r="D87" s="11"/>
@@ -4338,7 +4344,7 @@
       <c r="B88" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="C88" s="13" t="s">
+      <c r="C88" s="16" t="s">
         <v>170</v>
       </c>
       <c r="D88" s="11"/>
@@ -4349,7 +4355,7 @@
       <c r="B89" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="C89" s="13" t="s">
+      <c r="C89" s="16" t="s">
         <v>172</v>
       </c>
       <c r="D89" s="11"/>
@@ -4360,7 +4366,7 @@
       <c r="B90" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="C90" s="13" t="s">
+      <c r="C90" s="16" t="s">
         <v>174</v>
       </c>
       <c r="D90" s="11"/>
@@ -4380,7 +4386,7 @@
       <c r="B92" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="C92" s="13" t="s">
+      <c r="C92" s="16" t="s">
         <v>177</v>
       </c>
       <c r="D92" s="11"/>
@@ -4391,7 +4397,7 @@
       <c r="B93" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="C93" s="13" t="s">
+      <c r="C93" s="16" t="s">
         <v>179</v>
       </c>
       <c r="D93" s="11"/>
@@ -4402,7 +4408,7 @@
       <c r="B94" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="C94" s="13" t="s">
+      <c r="C94" s="16" t="s">
         <v>181</v>
       </c>
       <c r="D94" s="11"/>
@@ -4413,7 +4419,7 @@
       <c r="B95" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="C95" s="13" t="s">
+      <c r="C95" s="16" t="s">
         <v>183</v>
       </c>
       <c r="D95" s="11"/>
@@ -4424,7 +4430,7 @@
       <c r="B96" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="C96" s="13" t="s">
+      <c r="C96" s="16" t="s">
         <v>185</v>
       </c>
       <c r="D96" s="11"/>
@@ -4435,7 +4441,7 @@
       <c r="B97" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="C97" s="13" t="s">
+      <c r="C97" s="16" t="s">
         <v>187</v>
       </c>
       <c r="D97" s="11"/>
@@ -4446,7 +4452,7 @@
       <c r="B98" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="C98" s="13" t="s">
+      <c r="C98" s="16" t="s">
         <v>189</v>
       </c>
       <c r="D98" s="11"/>
@@ -4457,7 +4463,7 @@
       <c r="B99" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="C99" s="13" t="s">
+      <c r="C99" s="16" t="s">
         <v>191</v>
       </c>
       <c r="D99" s="11"/>
@@ -4468,7 +4474,7 @@
       <c r="B100" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="C100" s="13" t="s">
+      <c r="C100" s="16" t="s">
         <v>193</v>
       </c>
       <c r="D100" s="11"/>
@@ -4479,7 +4485,7 @@
       <c r="B101" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="C101" s="13" t="s">
+      <c r="C101" s="16" t="s">
         <v>195</v>
       </c>
       <c r="D101" s="11"/>
@@ -4490,7 +4496,7 @@
       <c r="B102" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="C102" s="13" t="s">
+      <c r="C102" s="16" t="s">
         <v>197</v>
       </c>
       <c r="D102" s="11"/>
@@ -4501,7 +4507,7 @@
       <c r="B103" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="C103" s="13" t="s">
+      <c r="C103" s="16" t="s">
         <v>199</v>
       </c>
       <c r="D103" s="11"/>
@@ -4512,7 +4518,7 @@
       <c r="B104" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="C104" s="13" t="s">
+      <c r="C104" s="16" t="s">
         <v>201</v>
       </c>
       <c r="D104" s="11"/>
@@ -4523,7 +4529,7 @@
       <c r="B105" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="C105" s="13" t="s">
+      <c r="C105" s="16" t="s">
         <v>203</v>
       </c>
       <c r="D105" s="11"/>
@@ -4534,7 +4540,7 @@
       <c r="B106" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="C106" s="13" t="s">
+      <c r="C106" s="16" t="s">
         <v>205</v>
       </c>
       <c r="D106" s="11"/>
@@ -4545,7 +4551,7 @@
       <c r="B107" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="C107" s="17" t="s">
+      <c r="C107" s="18" t="s">
         <v>207</v>
       </c>
       <c r="D107" s="11"/>
@@ -4556,7 +4562,7 @@
       <c r="B108" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="C108" s="17" t="s">
+      <c r="C108" s="18" t="s">
         <v>209</v>
       </c>
       <c r="D108" s="11"/>
@@ -4567,7 +4573,7 @@
       <c r="B109" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="C109" s="17" t="s">
+      <c r="C109" s="18" t="s">
         <v>211</v>
       </c>
       <c r="D109" s="11"/>
@@ -4578,7 +4584,7 @@
       <c r="B110" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="C110" s="17" t="s">
+      <c r="C110" s="18" t="s">
         <v>213</v>
       </c>
       <c r="D110" s="11"/>
@@ -4589,7 +4595,7 @@
       <c r="B111" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="C111" s="17" t="s">
+      <c r="C111" s="18" t="s">
         <v>215</v>
       </c>
       <c r="D111" s="11"/>
@@ -4600,7 +4606,7 @@
       <c r="B112" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="C112" s="17" t="s">
+      <c r="C112" s="18" t="s">
         <v>217</v>
       </c>
       <c r="D112" s="11"/>
@@ -4611,7 +4617,7 @@
       <c r="B113" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="C113" s="17" t="s">
+      <c r="C113" s="18" t="s">
         <v>219</v>
       </c>
       <c r="D113" s="11"/>
@@ -4631,7 +4637,7 @@
       <c r="B115" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="C115" s="13" t="s">
+      <c r="C115" s="16" t="s">
         <v>222</v>
       </c>
       <c r="D115" s="11"/>
@@ -4642,7 +4648,7 @@
       <c r="B116" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="C116" s="13" t="s">
+      <c r="C116" s="16" t="s">
         <v>224</v>
       </c>
       <c r="D116" s="11"/>
@@ -4653,7 +4659,7 @@
       <c r="B117" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="C117" s="13" t="s">
+      <c r="C117" s="16" t="s">
         <v>226</v>
       </c>
       <c r="D117" s="11"/>
@@ -4673,7 +4679,7 @@
       <c r="B119" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="C119" s="13" t="s">
+      <c r="C119" s="16" t="s">
         <v>229</v>
       </c>
       <c r="D119" s="11"/>
@@ -4693,7 +4699,7 @@
       <c r="B121" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="C121" s="13" t="s">
+      <c r="C121" s="16" t="s">
         <v>232</v>
       </c>
       <c r="D121" s="11"/>
@@ -4704,7 +4710,7 @@
       <c r="B122" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="C122" s="13" t="s">
+      <c r="C122" s="16" t="s">
         <v>234</v>
       </c>
       <c r="D122" s="11"/>
@@ -4751,7 +4757,7 @@
       <c r="B127" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="C127" s="13" t="s">
+      <c r="C127" s="16" t="s">
         <v>240</v>
       </c>
       <c r="D127" s="11"/>
@@ -4762,7 +4768,7 @@
       <c r="B128" s="8" t="s">
         <v>241</v>
       </c>
-      <c r="C128" s="13" t="s">
+      <c r="C128" s="16" t="s">
         <v>242</v>
       </c>
       <c r="D128" s="11"/>
@@ -4773,7 +4779,7 @@
       <c r="B129" s="8" t="s">
         <v>243</v>
       </c>
-      <c r="C129" s="13" t="s">
+      <c r="C129" s="16" t="s">
         <v>244</v>
       </c>
       <c r="D129" s="11"/>
@@ -4784,7 +4790,7 @@
       <c r="B130" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="C130" s="13" t="s">
+      <c r="C130" s="16" t="s">
         <v>246</v>
       </c>
       <c r="D130" s="11"/>
@@ -4804,7 +4810,7 @@
       <c r="B132" s="8" t="s">
         <v>248</v>
       </c>
-      <c r="C132" s="13" t="s">
+      <c r="C132" s="16" t="s">
         <v>249</v>
       </c>
       <c r="D132" s="11"/>
@@ -4815,7 +4821,7 @@
       <c r="B133" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="C133" s="13" t="s">
+      <c r="C133" s="16" t="s">
         <v>251</v>
       </c>
       <c r="D133" s="11"/>
@@ -4826,7 +4832,7 @@
       <c r="B134" s="8" t="s">
         <v>252</v>
       </c>
-      <c r="C134" s="13" t="s">
+      <c r="C134" s="16" t="s">
         <v>253</v>
       </c>
       <c r="D134" s="11"/>
@@ -4855,7 +4861,7 @@
       <c r="B137" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="C137" s="13" t="s">
+      <c r="C137" s="16" t="s">
         <v>257</v>
       </c>
       <c r="D137" s="11"/>
@@ -4920,7 +4926,7 @@
       <c r="B144" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="C144" s="13" t="s">
+      <c r="C144" s="16" t="s">
         <v>265</v>
       </c>
       <c r="E144" s="11"/>
@@ -4939,7 +4945,7 @@
       <c r="B146" s="27" t="s">
         <v>267</v>
       </c>
-      <c r="C146" s="13" t="s">
+      <c r="C146" s="16" t="s">
         <v>268</v>
       </c>
       <c r="D146" s="11"/>
@@ -4977,7 +4983,7 @@
       <c r="B150" s="8" t="s">
         <v>272</v>
       </c>
-      <c r="C150" s="13" t="s">
+      <c r="C150" s="16" t="s">
         <v>273</v>
       </c>
       <c r="D150" s="11"/>
@@ -5051,7 +5057,7 @@
       <c r="B158" s="8" t="s">
         <v>281</v>
       </c>
-      <c r="C158" s="13" t="s">
+      <c r="C158" s="16" t="s">
         <v>282</v>
       </c>
       <c r="E158" s="11"/>
@@ -5070,7 +5076,7 @@
       <c r="B160" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="C160" s="13" t="s">
+      <c r="C160" s="16" t="s">
         <v>285</v>
       </c>
       <c r="D160" s="11"/>
@@ -5081,7 +5087,7 @@
       <c r="B161" s="8" t="s">
         <v>286</v>
       </c>
-      <c r="C161" s="13" t="s">
+      <c r="C161" s="16" t="s">
         <v>287</v>
       </c>
       <c r="D161" s="11"/>
@@ -5092,7 +5098,7 @@
       <c r="B162" s="8" t="s">
         <v>288</v>
       </c>
-      <c r="C162" s="13" t="s">
+      <c r="C162" s="16" t="s">
         <v>289</v>
       </c>
       <c r="D162" s="11"/>
@@ -5103,7 +5109,7 @@
       <c r="B163" s="8" t="s">
         <v>290</v>
       </c>
-      <c r="C163" s="13" t="s">
+      <c r="C163" s="16" t="s">
         <v>291</v>
       </c>
       <c r="D163" s="11"/>
@@ -5132,7 +5138,7 @@
       <c r="B166" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="C166" s="13" t="s">
+      <c r="C166" s="16" t="s">
         <v>295</v>
       </c>
       <c r="D166" s="11"/>
@@ -5143,7 +5149,7 @@
       <c r="B167" s="8" t="s">
         <v>296</v>
       </c>
-      <c r="C167" s="13" t="s">
+      <c r="C167" s="16" t="s">
         <v>297</v>
       </c>
       <c r="D167" s="11"/>
@@ -5154,7 +5160,7 @@
       <c r="B168" s="8" t="s">
         <v>298</v>
       </c>
-      <c r="C168" s="13" t="s">
+      <c r="C168" s="16" t="s">
         <v>299</v>
       </c>
       <c r="D168" s="11"/>
@@ -5165,7 +5171,7 @@
       <c r="B169" s="8" t="s">
         <v>300</v>
       </c>
-      <c r="C169" s="13" t="s">
+      <c r="C169" s="16" t="s">
         <v>301</v>
       </c>
       <c r="D169" s="11"/>
@@ -5176,7 +5182,7 @@
       <c r="B170" s="8" t="s">
         <v>302</v>
       </c>
-      <c r="C170" s="13" t="s">
+      <c r="C170" s="16" t="s">
         <v>303</v>
       </c>
       <c r="D170" s="11"/>
@@ -5187,7 +5193,7 @@
       <c r="B171" s="8" t="s">
         <v>304</v>
       </c>
-      <c r="C171" s="13" t="s">
+      <c r="C171" s="16" t="s">
         <v>305</v>
       </c>
       <c r="D171" s="11"/>
@@ -5207,7 +5213,7 @@
       <c r="B173" s="8" t="s">
         <v>307</v>
       </c>
-      <c r="C173" s="13" t="s">
+      <c r="C173" s="16" t="s">
         <v>308</v>
       </c>
       <c r="D173" s="11"/>
@@ -5218,7 +5224,7 @@
       <c r="B174" s="8" t="s">
         <v>309</v>
       </c>
-      <c r="C174" s="13" t="s">
+      <c r="C174" s="16" t="s">
         <v>310</v>
       </c>
       <c r="D174" s="11"/>
@@ -5229,7 +5235,7 @@
       <c r="B175" s="8" t="s">
         <v>311</v>
       </c>
-      <c r="C175" s="13" t="s">
+      <c r="C175" s="16" t="s">
         <v>312</v>
       </c>
       <c r="D175" s="11"/>
@@ -5240,7 +5246,7 @@
       <c r="B176" s="8" t="s">
         <v>313</v>
       </c>
-      <c r="C176" s="13" t="s">
+      <c r="C176" s="16" t="s">
         <v>314</v>
       </c>
       <c r="E176" s="11"/>
@@ -5277,13 +5283,13 @@
       <c r="B180" s="8" t="s">
         <v>318</v>
       </c>
-      <c r="C180" s="13" t="s">
+      <c r="C180" s="16" t="s">
         <v>319</v>
       </c>
-      <c r="D180" s="13" t="s">
+      <c r="D180" s="16" t="s">
         <v>320</v>
       </c>
-      <c r="E180" s="13" t="s">
+      <c r="E180" s="16" t="s">
         <v>321</v>
       </c>
     </row>
@@ -5292,10 +5298,10 @@
       <c r="B181" s="8" t="s">
         <v>322</v>
       </c>
-      <c r="C181" s="13" t="s">
+      <c r="C181" s="16" t="s">
         <v>323</v>
       </c>
-      <c r="D181" s="13" t="s">
+      <c r="D181" s="16" t="s">
         <v>324</v>
       </c>
       <c r="E181" s="11"/>
@@ -5305,7 +5311,7 @@
       <c r="B182" s="8" t="s">
         <v>325</v>
       </c>
-      <c r="C182" s="13" t="s">
+      <c r="C182" s="16" t="s">
         <v>326</v>
       </c>
       <c r="D182" s="11"/>
@@ -5316,7 +5322,7 @@
       <c r="B183" s="8" t="s">
         <v>327</v>
       </c>
-      <c r="C183" s="13" t="s">
+      <c r="C183" s="16" t="s">
         <v>328</v>
       </c>
       <c r="D183" s="11"/>
@@ -5327,7 +5333,7 @@
       <c r="B184" s="8" t="s">
         <v>329</v>
       </c>
-      <c r="C184" s="13" t="s">
+      <c r="C184" s="16" t="s">
         <v>330</v>
       </c>
       <c r="D184" s="11"/>
@@ -5347,7 +5353,7 @@
       <c r="B186" s="8" t="s">
         <v>332</v>
       </c>
-      <c r="C186" s="13" t="s">
+      <c r="C186" s="16" t="s">
         <v>333</v>
       </c>
       <c r="D186" s="11"/>
@@ -5358,7 +5364,7 @@
       <c r="B187" s="8" t="s">
         <v>334</v>
       </c>
-      <c r="C187" s="13" t="s">
+      <c r="C187" s="16" t="s">
         <v>335</v>
       </c>
       <c r="D187" s="11"/>
@@ -5369,7 +5375,7 @@
       <c r="B188" s="8" t="s">
         <v>336</v>
       </c>
-      <c r="C188" s="13" t="s">
+      <c r="C188" s="16" t="s">
         <v>337</v>
       </c>
       <c r="D188" s="11"/>
@@ -5380,7 +5386,7 @@
       <c r="B189" s="8" t="s">
         <v>338</v>
       </c>
-      <c r="C189" s="13" t="s">
+      <c r="C189" s="16" t="s">
         <v>339</v>
       </c>
       <c r="D189" s="11"/>
@@ -5391,7 +5397,7 @@
       <c r="B190" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="C190" s="13" t="s">
+      <c r="C190" s="16" t="s">
         <v>341</v>
       </c>
       <c r="D190" s="11"/>
@@ -5411,7 +5417,7 @@
       <c r="B192" s="8" t="s">
         <v>343</v>
       </c>
-      <c r="C192" s="13" t="s">
+      <c r="C192" s="16" t="s">
         <v>344</v>
       </c>
       <c r="D192" s="11"/>
@@ -5422,7 +5428,7 @@
       <c r="B193" s="8" t="s">
         <v>345</v>
       </c>
-      <c r="C193" s="13" t="s">
+      <c r="C193" s="16" t="s">
         <v>346</v>
       </c>
       <c r="D193" s="11"/>
@@ -5433,7 +5439,7 @@
       <c r="B194" s="8" t="s">
         <v>347</v>
       </c>
-      <c r="C194" s="13" t="s">
+      <c r="C194" s="16" t="s">
         <v>346</v>
       </c>
       <c r="D194" s="11"/>
@@ -5444,7 +5450,7 @@
       <c r="B195" s="8" t="s">
         <v>348</v>
       </c>
-      <c r="C195" s="13" t="s">
+      <c r="C195" s="16" t="s">
         <v>349</v>
       </c>
       <c r="D195" s="11"/>
@@ -5455,7 +5461,7 @@
       <c r="B196" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="C196" s="13" t="s">
+      <c r="C196" s="16" t="s">
         <v>351</v>
       </c>
       <c r="D196" s="11"/>
@@ -5466,7 +5472,7 @@
       <c r="B197" s="8" t="s">
         <v>352</v>
       </c>
-      <c r="C197" s="13" t="s">
+      <c r="C197" s="16" t="s">
         <v>353</v>
       </c>
       <c r="D197" s="11"/>
@@ -5477,7 +5483,7 @@
       <c r="B198" s="8" t="s">
         <v>354</v>
       </c>
-      <c r="C198" s="13" t="s">
+      <c r="C198" s="16" t="s">
         <v>355</v>
       </c>
       <c r="D198" s="11"/>
@@ -5497,10 +5503,10 @@
       <c r="B200" s="8" t="s">
         <v>357</v>
       </c>
-      <c r="C200" s="13" t="s">
+      <c r="C200" s="16" t="s">
         <v>358</v>
       </c>
-      <c r="D200" s="13" t="s">
+      <c r="D200" s="16" t="s">
         <v>359</v>
       </c>
       <c r="E200" s="11"/>
@@ -5510,7 +5516,7 @@
       <c r="B201" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="C201" s="13" t="s">
+      <c r="C201" s="16" t="s">
         <v>224</v>
       </c>
       <c r="D201" s="11"/>
@@ -5521,7 +5527,7 @@
       <c r="B202" s="8" t="s">
         <v>360</v>
       </c>
-      <c r="C202" s="13" t="s">
+      <c r="C202" s="16" t="s">
         <v>361</v>
       </c>
       <c r="D202" s="11"/>
@@ -5532,7 +5538,7 @@
       <c r="B203" s="8" t="s">
         <v>362</v>
       </c>
-      <c r="C203" s="13" t="s">
+      <c r="C203" s="16" t="s">
         <v>363</v>
       </c>
       <c r="D203" s="11"/>
@@ -5552,7 +5558,7 @@
       <c r="B205" s="8" t="s">
         <v>365</v>
       </c>
-      <c r="C205" s="13" t="s">
+      <c r="C205" s="16" t="s">
         <v>366</v>
       </c>
       <c r="D205" s="11"/>
@@ -5563,7 +5569,7 @@
       <c r="B206" s="8" t="s">
         <v>367</v>
       </c>
-      <c r="C206" s="13" t="s">
+      <c r="C206" s="16" t="s">
         <v>368</v>
       </c>
       <c r="D206" s="11"/>
@@ -5574,13 +5580,13 @@
       <c r="B207" s="8" t="s">
         <v>369</v>
       </c>
-      <c r="C207" s="13" t="s">
+      <c r="C207" s="16" t="s">
         <v>370</v>
       </c>
-      <c r="D207" s="13" t="s">
+      <c r="D207" s="16" t="s">
         <v>371</v>
       </c>
-      <c r="E207" s="13" t="s">
+      <c r="E207" s="16" t="s">
         <v>372</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add InsertInterval class to handle interval insertion and merging
</commit_message>
<xml_diff>
--- a/DSA patterns Cheat Sheet.xlsx
+++ b/DSA patterns Cheat Sheet.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="373">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3984,11 +3984,14 @@
       <c r="B54" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C54" s="16" t="s">
+      <c r="C54" s="13" t="s">
         <v>107</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="11"/>
+      <c r="F54" s="12" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="55" customHeight="1" spans="1:6">
       <c r="A55" s="8"/>

</xml_diff>